<commit_message>
save: add temporary generate sf1 feature files
</commit_message>
<xml_diff>
--- a/backend/forms/SF1_template.xlsx
+++ b/backend/forms/SF1_template.xlsx
@@ -1733,7 +1733,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AU1000"/>
+  <dimension ref="A1:AU999"/>
   <sheetFormatPr defaultColWidth="12.6285714285714" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.1333333333333" customWidth="1"/>
@@ -4573,52 +4573,88 @@
       <c r="AT57" s="7"/>
       <c r="AU57" s="2"/>
     </row>
-    <row r="58" ht="27.75" customHeight="1" spans="1:47">
-      <c r="A58" s="20"/>
+    <row r="58" ht="19.5" customHeight="1" spans="1:47">
+      <c r="A58" s="26"/>
       <c r="B58" s="7"/>
-      <c r="C58" s="20"/>
+      <c r="C58" s="20" t="s">
+        <v>36</v>
+      </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
       <c r="F58" s="7"/>
-      <c r="G58" s="21"/>
-      <c r="H58" s="22"/>
+      <c r="G58" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="H58" s="28" t="s">
+        <v>35</v>
+      </c>
       <c r="I58" s="7"/>
-      <c r="J58" s="23"/>
+      <c r="J58" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="K58" s="7"/>
-      <c r="L58" s="20"/>
+      <c r="L58" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="M58" s="7"/>
-      <c r="N58" s="24"/>
-      <c r="O58" s="24"/>
-      <c r="P58" s="20"/>
+      <c r="N58" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="O58" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="P58" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="Q58" s="7"/>
-      <c r="R58" s="20"/>
+      <c r="R58" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="S58" s="6"/>
       <c r="T58" s="7"/>
-      <c r="U58" s="20"/>
+      <c r="U58" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="V58" s="7"/>
-      <c r="W58" s="20"/>
+      <c r="W58" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="X58" s="6"/>
       <c r="Y58" s="6"/>
       <c r="Z58" s="6"/>
       <c r="AA58" s="7"/>
-      <c r="AB58" s="20"/>
+      <c r="AB58" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="AC58" s="6"/>
       <c r="AD58" s="6"/>
       <c r="AE58" s="7"/>
-      <c r="AF58" s="20"/>
+      <c r="AF58" s="29" t="s">
+        <v>35</v>
+      </c>
       <c r="AG58" s="6"/>
       <c r="AH58" s="6"/>
       <c r="AI58" s="6"/>
       <c r="AJ58" s="7"/>
-      <c r="AK58" s="20"/>
+      <c r="AK58" s="31" t="s">
+        <v>35</v>
+      </c>
       <c r="AL58" s="6"/>
       <c r="AM58" s="6"/>
       <c r="AN58" s="7"/>
-      <c r="AO58" s="24"/>
-      <c r="AP58" s="25"/>
+      <c r="AO58" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="AP58" s="31" t="s">
+        <v>35</v>
+      </c>
       <c r="AQ58" s="7"/>
-      <c r="AR58" s="21"/>
-      <c r="AS58" s="23"/>
+      <c r="AR58" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="AS58" s="31" t="s">
+        <v>35</v>
+      </c>
       <c r="AT58" s="7"/>
       <c r="AU58" s="2"/>
     </row>
@@ -4626,7 +4662,7 @@
       <c r="A59" s="26"/>
       <c r="B59" s="7"/>
       <c r="C59" s="20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
@@ -4707,219 +4743,160 @@
       <c r="AT59" s="7"/>
       <c r="AU59" s="2"/>
     </row>
-    <row r="60" ht="19.5" customHeight="1" spans="1:47">
-      <c r="A60" s="26"/>
-      <c r="B60" s="7"/>
-      <c r="C60" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="D60" s="6"/>
-      <c r="E60" s="6"/>
-      <c r="F60" s="7"/>
-      <c r="G60" s="27" t="s">
+    <row r="60" customHeight="1" spans="1:47">
+      <c r="A60" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="T60" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="H60" s="28" t="s">
+      <c r="V60" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="I60" s="7"/>
-      <c r="J60" s="29" t="s">
+      <c r="AT60" s="2"/>
+      <c r="AU60" s="2"/>
+    </row>
+    <row r="61" customHeight="1" spans="1:47">
+      <c r="A61" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="B61" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C61" s="7"/>
+      <c r="D61" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="J61" s="6"/>
+      <c r="K61" s="6"/>
+      <c r="L61" s="7"/>
+      <c r="M61" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="N61" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="O61" s="6"/>
+      <c r="P61" s="6"/>
+      <c r="Q61" s="6"/>
+      <c r="R61" s="6"/>
+      <c r="S61" s="7"/>
+      <c r="V61" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="W61" s="7"/>
+      <c r="X61" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y61" s="6"/>
+      <c r="Z61" s="7"/>
+      <c r="AA61" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB61" s="7"/>
+      <c r="AC61" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="K60" s="7"/>
-      <c r="L60" s="29" t="s">
+      <c r="AE61" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="AL61" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="M60" s="7"/>
-      <c r="N60" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="O60" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="P60" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q60" s="7"/>
-      <c r="R60" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="S60" s="6"/>
-      <c r="T60" s="7"/>
-      <c r="U60" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="V60" s="7"/>
-      <c r="W60" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="X60" s="6"/>
-      <c r="Y60" s="6"/>
-      <c r="Z60" s="6"/>
-      <c r="AA60" s="7"/>
-      <c r="AB60" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC60" s="6"/>
-      <c r="AD60" s="6"/>
-      <c r="AE60" s="7"/>
-      <c r="AF60" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG60" s="6"/>
-      <c r="AH60" s="6"/>
-      <c r="AI60" s="6"/>
-      <c r="AJ60" s="7"/>
-      <c r="AK60" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL60" s="6"/>
-      <c r="AM60" s="6"/>
-      <c r="AN60" s="7"/>
-      <c r="AO60" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AP60" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AQ60" s="7"/>
-      <c r="AR60" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AS60" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AT60" s="7"/>
-      <c r="AU60" s="2"/>
-    </row>
-    <row r="61" customHeight="1" spans="1:47">
-      <c r="A61" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="T61" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="V61" s="34" t="s">
-        <v>35</v>
+      <c r="AN61" s="37" t="s">
+        <v>46</v>
       </c>
       <c r="AT61" s="2"/>
       <c r="AU61" s="2"/>
     </row>
-    <row r="62" customHeight="1" spans="1:47">
-      <c r="A62" s="35" t="s">
-        <v>39</v>
-      </c>
-      <c r="B62" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C62" s="7"/>
-      <c r="D62" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="E62" s="6"/>
-      <c r="F62" s="6"/>
-      <c r="G62" s="6"/>
-      <c r="H62" s="7"/>
-      <c r="I62" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="J62" s="6"/>
-      <c r="K62" s="6"/>
-      <c r="L62" s="7"/>
-      <c r="M62" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="N62" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="O62" s="6"/>
-      <c r="P62" s="6"/>
-      <c r="Q62" s="6"/>
-      <c r="R62" s="6"/>
-      <c r="S62" s="7"/>
-      <c r="V62" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="W62" s="7"/>
-      <c r="X62" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="Y62" s="6"/>
-      <c r="Z62" s="7"/>
-      <c r="AA62" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="AB62" s="7"/>
-      <c r="AC62" s="33" t="s">
+    <row r="62" ht="13.5" customHeight="1" spans="1:47">
+      <c r="A62" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="B62" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="C62" s="9"/>
+      <c r="D62" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="E62" s="10"/>
+      <c r="F62" s="10"/>
+      <c r="G62" s="10"/>
+      <c r="H62" s="9"/>
+      <c r="I62" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="J62" s="10"/>
+      <c r="K62" s="10"/>
+      <c r="L62" s="9"/>
+      <c r="M62" s="41" t="s">
+        <v>51</v>
+      </c>
+      <c r="N62" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="O62" s="10"/>
+      <c r="P62" s="10"/>
+      <c r="Q62" s="10"/>
+      <c r="R62" s="10"/>
+      <c r="S62" s="9"/>
+      <c r="V62" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="W62" s="9"/>
+      <c r="X62" s="8">
+        <v>25</v>
+      </c>
+      <c r="Y62" s="10"/>
+      <c r="Z62" s="9"/>
+      <c r="AA62" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="AE62" s="37" t="s">
-        <v>45</v>
-      </c>
-      <c r="AL62" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="AN62" s="37" t="s">
-        <v>46</v>
+      <c r="AB62" s="9"/>
+      <c r="AE62" s="42" t="s">
+        <v>54</v>
+      </c>
+      <c r="AN62" s="43" t="s">
+        <v>55</v>
       </c>
       <c r="AT62" s="2"/>
       <c r="AU62" s="2"/>
     </row>
-    <row r="63" ht="13.5" customHeight="1" spans="1:47">
-      <c r="A63" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="B63" s="39" t="s">
-        <v>48</v>
-      </c>
-      <c r="C63" s="9"/>
-      <c r="D63" s="40" t="s">
-        <v>49</v>
-      </c>
-      <c r="E63" s="10"/>
-      <c r="F63" s="10"/>
-      <c r="G63" s="10"/>
-      <c r="H63" s="9"/>
-      <c r="I63" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="J63" s="10"/>
-      <c r="K63" s="10"/>
-      <c r="L63" s="9"/>
-      <c r="M63" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="N63" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="O63" s="10"/>
-      <c r="P63" s="10"/>
-      <c r="Q63" s="10"/>
-      <c r="R63" s="10"/>
-      <c r="S63" s="9"/>
-      <c r="V63" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="W63" s="9"/>
-      <c r="X63" s="8">
-        <v>25</v>
-      </c>
-      <c r="Y63" s="10"/>
-      <c r="Z63" s="9"/>
-      <c r="AA63" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB63" s="9"/>
-      <c r="AE63" s="42" t="s">
-        <v>54</v>
-      </c>
-      <c r="AN63" s="43" t="s">
-        <v>55</v>
-      </c>
+    <row r="63" ht="0.75" customHeight="1" spans="1:47">
+      <c r="A63" s="44"/>
+      <c r="B63" s="45"/>
+      <c r="C63" s="46"/>
+      <c r="D63" s="45"/>
+      <c r="H63" s="46"/>
+      <c r="I63" s="45"/>
+      <c r="L63" s="46"/>
+      <c r="M63" s="44"/>
+      <c r="N63" s="45"/>
+      <c r="S63" s="46"/>
+      <c r="V63" s="45"/>
+      <c r="W63" s="46"/>
+      <c r="X63" s="45"/>
+      <c r="Z63" s="46"/>
+      <c r="AA63" s="45"/>
+      <c r="AB63" s="46"/>
+      <c r="AN63" s="2"/>
+      <c r="AO63" s="2"/>
+      <c r="AP63" s="2"/>
+      <c r="AQ63" s="2"/>
+      <c r="AR63" s="2"/>
+      <c r="AS63" s="2"/>
       <c r="AT63" s="2"/>
       <c r="AU63" s="2"/>
     </row>
-    <row r="64" ht="0.75" customHeight="1" spans="1:47">
+    <row r="64" ht="9.75" customHeight="1" spans="1:47">
       <c r="A64" s="44"/>
       <c r="B64" s="45"/>
       <c r="C64" s="46"/>
@@ -4930,18 +4907,23 @@
       <c r="M64" s="44"/>
       <c r="N64" s="45"/>
       <c r="S64" s="46"/>
-      <c r="V64" s="45"/>
-      <c r="W64" s="46"/>
-      <c r="X64" s="45"/>
-      <c r="Z64" s="46"/>
-      <c r="AA64" s="45"/>
-      <c r="AB64" s="46"/>
-      <c r="AN64" s="2"/>
-      <c r="AO64" s="2"/>
-      <c r="AP64" s="2"/>
-      <c r="AQ64" s="2"/>
-      <c r="AR64" s="2"/>
-      <c r="AS64" s="2"/>
+      <c r="V64" s="15"/>
+      <c r="W64" s="16"/>
+      <c r="X64" s="15"/>
+      <c r="Y64" s="17"/>
+      <c r="Z64" s="16"/>
+      <c r="AA64" s="15"/>
+      <c r="AB64" s="16"/>
+      <c r="AE64" s="47"/>
+      <c r="AF64" s="47"/>
+      <c r="AG64" s="47"/>
+      <c r="AH64" s="47"/>
+      <c r="AI64" s="47"/>
+      <c r="AJ64" s="47"/>
+      <c r="AK64" s="47"/>
+      <c r="AN64" s="48" t="s">
+        <v>56</v>
+      </c>
       <c r="AT64" s="2"/>
       <c r="AU64" s="2"/>
     </row>
@@ -4956,22 +4938,21 @@
       <c r="M65" s="44"/>
       <c r="N65" s="45"/>
       <c r="S65" s="46"/>
-      <c r="V65" s="15"/>
-      <c r="W65" s="16"/>
-      <c r="X65" s="15"/>
-      <c r="Y65" s="17"/>
-      <c r="Z65" s="16"/>
-      <c r="AA65" s="15"/>
-      <c r="AB65" s="16"/>
-      <c r="AE65" s="47"/>
-      <c r="AF65" s="47"/>
-      <c r="AG65" s="47"/>
-      <c r="AH65" s="47"/>
-      <c r="AI65" s="47"/>
-      <c r="AJ65" s="47"/>
-      <c r="AK65" s="47"/>
-      <c r="AN65" s="48" t="s">
-        <v>56</v>
+      <c r="V65" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="W65" s="9"/>
+      <c r="X65" s="8">
+        <v>26</v>
+      </c>
+      <c r="Y65" s="10"/>
+      <c r="Z65" s="9"/>
+      <c r="AA65" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB65" s="9"/>
+      <c r="AE65" s="48" t="s">
+        <v>58</v>
       </c>
       <c r="AT65" s="2"/>
       <c r="AU65" s="2"/>
@@ -4987,21 +4968,18 @@
       <c r="M66" s="44"/>
       <c r="N66" s="45"/>
       <c r="S66" s="46"/>
-      <c r="V66" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="W66" s="9"/>
-      <c r="X66" s="8">
-        <v>26</v>
-      </c>
-      <c r="Y66" s="10"/>
-      <c r="Z66" s="9"/>
-      <c r="AA66" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB66" s="9"/>
-      <c r="AE66" s="48" t="s">
-        <v>58</v>
+      <c r="V66" s="15"/>
+      <c r="W66" s="16"/>
+      <c r="X66" s="15"/>
+      <c r="Y66" s="17"/>
+      <c r="Z66" s="16"/>
+      <c r="AA66" s="15"/>
+      <c r="AB66" s="16"/>
+      <c r="AN66" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="AQ66" s="49" t="s">
+        <v>60</v>
       </c>
       <c r="AT66" s="2"/>
       <c r="AU66" s="2"/>
@@ -5017,95 +4995,115 @@
       <c r="M67" s="44"/>
       <c r="N67" s="45"/>
       <c r="S67" s="46"/>
-      <c r="V67" s="15"/>
-      <c r="W67" s="16"/>
-      <c r="X67" s="15"/>
-      <c r="Y67" s="17"/>
-      <c r="Z67" s="16"/>
-      <c r="AA67" s="15"/>
-      <c r="AB67" s="16"/>
-      <c r="AN67" s="49" t="s">
+      <c r="V67" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="W67" s="9"/>
+      <c r="X67" s="8">
+        <v>51</v>
+      </c>
+      <c r="Y67" s="10"/>
+      <c r="Z67" s="9"/>
+      <c r="AA67" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB67" s="9"/>
+      <c r="AE67" s="49" t="s">
         <v>59</v>
       </c>
-      <c r="AQ67" s="49" t="s">
+      <c r="AI67" s="49" t="s">
         <v>60</v>
       </c>
+      <c r="AN67" s="47"/>
+      <c r="AO67" s="47"/>
+      <c r="AP67" s="47"/>
+      <c r="AQ67" s="47"/>
+      <c r="AR67" s="47"/>
+      <c r="AS67" s="47"/>
       <c r="AT67" s="2"/>
       <c r="AU67" s="2"/>
     </row>
-    <row r="68" ht="9.75" customHeight="1" spans="1:47">
-      <c r="A68" s="44"/>
-      <c r="B68" s="45"/>
-      <c r="C68" s="46"/>
-      <c r="D68" s="45"/>
-      <c r="H68" s="46"/>
-      <c r="I68" s="45"/>
-      <c r="L68" s="46"/>
-      <c r="M68" s="44"/>
-      <c r="N68" s="45"/>
-      <c r="S68" s="46"/>
-      <c r="V68" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="W68" s="9"/>
-      <c r="X68" s="8">
-        <v>51</v>
-      </c>
-      <c r="Y68" s="10"/>
-      <c r="Z68" s="9"/>
-      <c r="AA68" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB68" s="9"/>
-      <c r="AE68" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="AI68" s="49" t="s">
-        <v>60</v>
-      </c>
-      <c r="AN68" s="47"/>
-      <c r="AO68" s="47"/>
-      <c r="AP68" s="47"/>
-      <c r="AQ68" s="47"/>
-      <c r="AR68" s="47"/>
-      <c r="AS68" s="47"/>
+    <row r="68" customHeight="1" spans="1:47">
+      <c r="A68" s="18"/>
+      <c r="B68" s="15"/>
+      <c r="C68" s="16"/>
+      <c r="D68" s="15"/>
+      <c r="E68" s="17"/>
+      <c r="F68" s="17"/>
+      <c r="G68" s="17"/>
+      <c r="H68" s="16"/>
+      <c r="I68" s="15"/>
+      <c r="J68" s="17"/>
+      <c r="K68" s="17"/>
+      <c r="L68" s="16"/>
+      <c r="M68" s="18"/>
+      <c r="N68" s="15"/>
+      <c r="O68" s="17"/>
+      <c r="P68" s="17"/>
+      <c r="Q68" s="17"/>
+      <c r="R68" s="17"/>
+      <c r="S68" s="16"/>
+      <c r="V68" s="15"/>
+      <c r="W68" s="16"/>
+      <c r="X68" s="15"/>
+      <c r="Y68" s="17"/>
+      <c r="Z68" s="16"/>
+      <c r="AA68" s="15"/>
+      <c r="AB68" s="16"/>
+      <c r="AE68" s="47"/>
+      <c r="AF68" s="47"/>
+      <c r="AG68" s="47"/>
+      <c r="AH68" s="47"/>
+      <c r="AI68" s="47"/>
+      <c r="AJ68" s="47"/>
+      <c r="AK68" s="47"/>
+      <c r="AN68" s="2"/>
+      <c r="AO68" s="2"/>
+      <c r="AP68" s="2"/>
+      <c r="AQ68" s="2"/>
+      <c r="AR68" s="2"/>
+      <c r="AS68" s="2"/>
       <c r="AT68" s="2"/>
       <c r="AU68" s="2"/>
     </row>
-    <row r="69" customHeight="1" spans="1:47">
-      <c r="A69" s="18"/>
-      <c r="B69" s="15"/>
-      <c r="C69" s="16"/>
-      <c r="D69" s="15"/>
-      <c r="E69" s="17"/>
-      <c r="F69" s="17"/>
-      <c r="G69" s="17"/>
-      <c r="H69" s="16"/>
-      <c r="I69" s="15"/>
-      <c r="J69" s="17"/>
-      <c r="K69" s="17"/>
-      <c r="L69" s="16"/>
-      <c r="M69" s="18"/>
-      <c r="N69" s="15"/>
-      <c r="O69" s="17"/>
-      <c r="P69" s="17"/>
-      <c r="Q69" s="17"/>
-      <c r="R69" s="17"/>
-      <c r="S69" s="16"/>
-      <c r="V69" s="15"/>
-      <c r="W69" s="16"/>
-      <c r="X69" s="15"/>
-      <c r="Y69" s="17"/>
-      <c r="Z69" s="16"/>
-      <c r="AA69" s="15"/>
-      <c r="AB69" s="16"/>
-      <c r="AE69" s="47"/>
-      <c r="AF69" s="47"/>
-      <c r="AG69" s="47"/>
-      <c r="AH69" s="47"/>
-      <c r="AI69" s="47"/>
-      <c r="AJ69" s="47"/>
-      <c r="AK69" s="47"/>
+    <row r="69" ht="9.75" customHeight="1" spans="1:47">
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2"/>
+      <c r="F69" s="2"/>
+      <c r="G69" s="2"/>
+      <c r="H69" s="2"/>
+      <c r="I69" s="2"/>
+      <c r="J69" s="2"/>
+      <c r="K69" s="2"/>
+      <c r="L69" s="2"/>
+      <c r="M69" s="2"/>
+      <c r="N69" s="2"/>
+      <c r="O69" s="2"/>
+      <c r="P69" s="2"/>
+      <c r="Q69" s="2"/>
+      <c r="R69" s="2"/>
+      <c r="S69" s="2"/>
+      <c r="T69" s="2"/>
+      <c r="U69" s="2"/>
+      <c r="V69" s="2"/>
+      <c r="W69" s="2"/>
+      <c r="X69" s="2"/>
+      <c r="Y69" s="2"/>
+      <c r="Z69" s="2"/>
+      <c r="AA69" s="2"/>
+      <c r="AB69" s="2"/>
+      <c r="AC69" s="2"/>
+      <c r="AD69" s="2"/>
+      <c r="AE69" s="2"/>
+      <c r="AF69" s="2"/>
+      <c r="AG69" s="2"/>
+      <c r="AH69" s="2"/>
+      <c r="AI69" s="2"/>
+      <c r="AJ69" s="2"/>
+      <c r="AK69" s="2"/>
       <c r="AN69" s="2"/>
       <c r="AO69" s="2"/>
       <c r="AP69" s="2"/>
@@ -5153,79 +5151,33 @@
       <c r="AI70" s="2"/>
       <c r="AJ70" s="2"/>
       <c r="AK70" s="2"/>
-      <c r="AN70" s="2"/>
-      <c r="AO70" s="2"/>
-      <c r="AP70" s="2"/>
-      <c r="AQ70" s="2"/>
-      <c r="AR70" s="2"/>
-      <c r="AS70" s="2"/>
+      <c r="AN70" s="50" t="s">
+        <v>62</v>
+      </c>
+      <c r="AO70" s="51"/>
+      <c r="AP70" s="51"/>
+      <c r="AQ70" s="51"/>
+      <c r="AR70" s="51"/>
+      <c r="AS70" s="51"/>
       <c r="AT70" s="2"/>
       <c r="AU70" s="2"/>
     </row>
-    <row r="71" ht="9.75" customHeight="1" spans="1:47">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
-      <c r="F71" s="2"/>
-      <c r="G71" s="2"/>
-      <c r="H71" s="2"/>
-      <c r="I71" s="2"/>
-      <c r="J71" s="2"/>
-      <c r="K71" s="2"/>
-      <c r="L71" s="2"/>
-      <c r="M71" s="2"/>
-      <c r="N71" s="2"/>
-      <c r="O71" s="2"/>
-      <c r="P71" s="2"/>
-      <c r="Q71" s="2"/>
-      <c r="R71" s="2"/>
-      <c r="S71" s="2"/>
-      <c r="T71" s="2"/>
-      <c r="U71" s="2"/>
-      <c r="V71" s="2"/>
-      <c r="W71" s="2"/>
-      <c r="X71" s="2"/>
-      <c r="Y71" s="2"/>
-      <c r="Z71" s="2"/>
-      <c r="AA71" s="2"/>
-      <c r="AB71" s="2"/>
-      <c r="AC71" s="2"/>
-      <c r="AD71" s="2"/>
-      <c r="AE71" s="2"/>
-      <c r="AF71" s="2"/>
-      <c r="AG71" s="2"/>
-      <c r="AH71" s="2"/>
-      <c r="AI71" s="2"/>
-      <c r="AJ71" s="2"/>
-      <c r="AK71" s="2"/>
-      <c r="AN71" s="50" t="s">
-        <v>62</v>
-      </c>
-      <c r="AO71" s="51"/>
-      <c r="AP71" s="51"/>
-      <c r="AQ71" s="51"/>
-      <c r="AR71" s="51"/>
-      <c r="AS71" s="51"/>
+    <row r="71" ht="19.5" customHeight="1" spans="1:47">
+      <c r="A71" s="52" t="s">
+        <v>63</v>
+      </c>
+      <c r="AL71" s="2"/>
+      <c r="AM71" s="2"/>
+      <c r="AN71" s="2"/>
+      <c r="AO71" s="2"/>
+      <c r="AP71" s="2"/>
+      <c r="AQ71" s="2"/>
+      <c r="AR71" s="2"/>
+      <c r="AS71" s="2"/>
       <c r="AT71" s="2"/>
       <c r="AU71" s="2"/>
     </row>
-    <row r="72" ht="19.5" customHeight="1" spans="1:47">
-      <c r="A72" s="52" t="s">
-        <v>63</v>
-      </c>
-      <c r="AL72" s="2"/>
-      <c r="AM72" s="2"/>
-      <c r="AN72" s="2"/>
-      <c r="AO72" s="2"/>
-      <c r="AP72" s="2"/>
-      <c r="AQ72" s="2"/>
-      <c r="AR72" s="2"/>
-      <c r="AS72" s="2"/>
-      <c r="AT72" s="2"/>
-      <c r="AU72" s="2"/>
-    </row>
+    <row r="72" ht="12.75" customHeight="1"/>
     <row r="73" ht="12.75" customHeight="1"/>
     <row r="74" ht="12.75" customHeight="1"/>
     <row r="75" ht="12.75" customHeight="1"/>
@@ -6153,9 +6105,8 @@
     <row r="997" ht="12.75" customHeight="1"/>
     <row r="998" ht="12.75" customHeight="1"/>
     <row r="999" ht="12.75" customHeight="1"/>
-    <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="832">
+  <mergeCells count="818">
     <mergeCell ref="A1:AT1"/>
     <mergeCell ref="A2:AT2"/>
     <mergeCell ref="A3:E3"/>
@@ -6925,37 +6876,23 @@
     <mergeCell ref="AK59:AN59"/>
     <mergeCell ref="AP59:AQ59"/>
     <mergeCell ref="AS59:AT59"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="C60:F60"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="J60:K60"/>
-    <mergeCell ref="L60:M60"/>
-    <mergeCell ref="P60:Q60"/>
-    <mergeCell ref="R60:T60"/>
-    <mergeCell ref="U60:V60"/>
-    <mergeCell ref="W60:AA60"/>
-    <mergeCell ref="AB60:AE60"/>
-    <mergeCell ref="AF60:AJ60"/>
-    <mergeCell ref="AK60:AN60"/>
-    <mergeCell ref="AP60:AQ60"/>
-    <mergeCell ref="AS60:AT60"/>
-    <mergeCell ref="A61:S61"/>
-    <mergeCell ref="V61:AS61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="D62:H62"/>
-    <mergeCell ref="I62:L62"/>
-    <mergeCell ref="N62:S62"/>
-    <mergeCell ref="V62:W62"/>
-    <mergeCell ref="X62:Z62"/>
-    <mergeCell ref="AA62:AB62"/>
-    <mergeCell ref="AE62:AK62"/>
+    <mergeCell ref="A60:S60"/>
+    <mergeCell ref="V60:AS60"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="D61:H61"/>
+    <mergeCell ref="I61:L61"/>
+    <mergeCell ref="N61:S61"/>
+    <mergeCell ref="V61:W61"/>
+    <mergeCell ref="X61:Z61"/>
+    <mergeCell ref="AA61:AB61"/>
+    <mergeCell ref="AE61:AK61"/>
+    <mergeCell ref="AN61:AS61"/>
     <mergeCell ref="AN62:AS62"/>
-    <mergeCell ref="AN63:AS63"/>
-    <mergeCell ref="AN71:AS71"/>
-    <mergeCell ref="A72:AK72"/>
-    <mergeCell ref="A63:A69"/>
+    <mergeCell ref="AN70:AS70"/>
+    <mergeCell ref="A71:AK71"/>
+    <mergeCell ref="A62:A68"/>
     <mergeCell ref="G5:G6"/>
-    <mergeCell ref="M63:M69"/>
+    <mergeCell ref="M62:M68"/>
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="O5:O6"/>
     <mergeCell ref="AR5:AR6"/>
@@ -6963,31 +6900,31 @@
     <mergeCell ref="J5:K6"/>
     <mergeCell ref="L5:M6"/>
     <mergeCell ref="AP5:AQ6"/>
-    <mergeCell ref="B63:C69"/>
-    <mergeCell ref="D63:H69"/>
-    <mergeCell ref="I63:L69"/>
-    <mergeCell ref="N63:S69"/>
-    <mergeCell ref="V63:W65"/>
-    <mergeCell ref="V66:W67"/>
-    <mergeCell ref="V68:W69"/>
-    <mergeCell ref="T61:U69"/>
-    <mergeCell ref="AE63:AK65"/>
-    <mergeCell ref="X66:Z67"/>
-    <mergeCell ref="AA66:AB67"/>
-    <mergeCell ref="AE66:AK67"/>
-    <mergeCell ref="AN67:AP68"/>
-    <mergeCell ref="AQ67:AS68"/>
-    <mergeCell ref="X63:Z65"/>
-    <mergeCell ref="X68:Z69"/>
-    <mergeCell ref="AA68:AB69"/>
-    <mergeCell ref="AE68:AH69"/>
-    <mergeCell ref="AC62:AD69"/>
-    <mergeCell ref="AL62:AM71"/>
-    <mergeCell ref="AA63:AB65"/>
-    <mergeCell ref="AI68:AK69"/>
     <mergeCell ref="A5:B6"/>
     <mergeCell ref="C5:F6"/>
-    <mergeCell ref="AN65:AS66"/>
+    <mergeCell ref="B62:C68"/>
+    <mergeCell ref="D62:H68"/>
+    <mergeCell ref="I62:L68"/>
+    <mergeCell ref="N62:S68"/>
+    <mergeCell ref="V62:W64"/>
+    <mergeCell ref="V65:W66"/>
+    <mergeCell ref="V67:W68"/>
+    <mergeCell ref="T60:U68"/>
+    <mergeCell ref="AE62:AK64"/>
+    <mergeCell ref="X65:Z66"/>
+    <mergeCell ref="AA65:AB66"/>
+    <mergeCell ref="AE65:AK66"/>
+    <mergeCell ref="AN66:AP67"/>
+    <mergeCell ref="AQ66:AS67"/>
+    <mergeCell ref="X62:Z64"/>
+    <mergeCell ref="X67:Z68"/>
+    <mergeCell ref="AA67:AB68"/>
+    <mergeCell ref="AE67:AH68"/>
+    <mergeCell ref="AC61:AD68"/>
+    <mergeCell ref="AL61:AM70"/>
+    <mergeCell ref="AA62:AB64"/>
+    <mergeCell ref="AI67:AK68"/>
+    <mergeCell ref="AN64:AS65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="14" fitToHeight="0" orientation="landscape"/>

</xml_diff>

<commit_message>
save: input and output reference
</commit_message>
<xml_diff>
--- a/backend/forms/SF1_template.xlsx
+++ b/backend/forms/SF1_template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="61">
   <si>
     <t>School Form 1 (SF 1) School Register</t>
   </si>
@@ -135,19 +135,10 @@
     <t>(Please refer to the legend on last page)</t>
   </si>
   <si>
-    <t>&lt;=== TOTAL MALE</t>
+    <t>List and Code of Indicators under REMARKS column</t>
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>&lt;=== TOTAL FEMALE</t>
-  </si>
-  <si>
-    <t>&lt;=== COMBINED</t>
-  </si>
-  <si>
-    <t>List and Code of Indicators under REMARKS column</t>
   </si>
   <si>
     <t>Indicator</t>
@@ -485,18 +476,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1002,7 +987,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1026,16 +1011,16 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="22" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="21" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1044,89 +1029,89 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1185,24 +1170,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1733,7 +1700,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AU999"/>
+  <dimension ref="A1:AU996"/>
   <sheetFormatPr defaultColWidth="12.6285714285714" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.1333333333333" customWidth="1"/>
@@ -3263,92 +3230,56 @@
       <c r="AT31" s="7"/>
       <c r="AU31" s="2"/>
     </row>
-    <row r="32" ht="19.5" customHeight="1" spans="1:47">
-      <c r="A32" s="26"/>
+    <row r="32" ht="37.5" customHeight="1" spans="1:47">
+      <c r="A32" s="20"/>
       <c r="B32" s="7"/>
-      <c r="C32" s="20" t="s">
-        <v>34</v>
-      </c>
+      <c r="C32" s="20"/>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="7"/>
-      <c r="G32" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="H32" s="28" t="s">
-        <v>35</v>
-      </c>
+      <c r="G32" s="21"/>
+      <c r="H32" s="22"/>
       <c r="I32" s="7"/>
-      <c r="J32" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="J32" s="23"/>
       <c r="K32" s="7"/>
-      <c r="L32" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="L32" s="20"/>
       <c r="M32" s="7"/>
-      <c r="N32" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="O32" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="P32" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="N32" s="24"/>
+      <c r="O32" s="24"/>
+      <c r="P32" s="20"/>
       <c r="Q32" s="7"/>
-      <c r="R32" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="R32" s="20"/>
       <c r="S32" s="6"/>
       <c r="T32" s="7"/>
-      <c r="U32" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="U32" s="20"/>
       <c r="V32" s="7"/>
-      <c r="W32" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="W32" s="20"/>
       <c r="X32" s="6"/>
       <c r="Y32" s="6"/>
       <c r="Z32" s="6"/>
       <c r="AA32" s="7"/>
-      <c r="AB32" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="AB32" s="20"/>
       <c r="AC32" s="6"/>
       <c r="AD32" s="6"/>
       <c r="AE32" s="7"/>
-      <c r="AF32" s="29" t="s">
-        <v>35</v>
-      </c>
+      <c r="AF32" s="20"/>
       <c r="AG32" s="6"/>
       <c r="AH32" s="6"/>
       <c r="AI32" s="6"/>
       <c r="AJ32" s="7"/>
-      <c r="AK32" s="31" t="s">
-        <v>35</v>
-      </c>
+      <c r="AK32" s="20"/>
       <c r="AL32" s="6"/>
       <c r="AM32" s="6"/>
       <c r="AN32" s="7"/>
-      <c r="AO32" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AP32" s="31" t="s">
-        <v>35</v>
-      </c>
+      <c r="AO32" s="24"/>
+      <c r="AP32" s="25"/>
       <c r="AQ32" s="7"/>
-      <c r="AR32" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AS32" s="31" t="s">
-        <v>35</v>
-      </c>
+      <c r="AR32" s="21"/>
+      <c r="AS32" s="23"/>
       <c r="AT32" s="7"/>
       <c r="AU32" s="2"/>
     </row>
-    <row r="33" ht="37.5" customHeight="1" spans="1:47">
+    <row r="33" ht="27.75" customHeight="1" spans="1:47">
       <c r="A33" s="20"/>
       <c r="B33" s="7"/>
       <c r="C33" s="20"/>
@@ -3446,7 +3377,7 @@
       <c r="AT34" s="7"/>
       <c r="AU34" s="2"/>
     </row>
-    <row r="35" ht="27.75" customHeight="1" spans="1:47">
+    <row r="35" ht="37.5" customHeight="1" spans="1:47">
       <c r="A35" s="20"/>
       <c r="B35" s="7"/>
       <c r="C35" s="20"/>
@@ -3495,7 +3426,7 @@
       <c r="AT35" s="7"/>
       <c r="AU35" s="2"/>
     </row>
-    <row r="36" ht="37.5" customHeight="1" spans="1:47">
+    <row r="36" ht="27.75" customHeight="1" spans="1:47">
       <c r="A36" s="20"/>
       <c r="B36" s="7"/>
       <c r="C36" s="20"/>
@@ -3544,7 +3475,7 @@
       <c r="AT36" s="7"/>
       <c r="AU36" s="2"/>
     </row>
-    <row r="37" ht="27.75" customHeight="1" spans="1:47">
+    <row r="37" ht="37.5" customHeight="1" spans="1:47">
       <c r="A37" s="20"/>
       <c r="B37" s="7"/>
       <c r="C37" s="20"/>
@@ -3593,7 +3524,7 @@
       <c r="AT37" s="7"/>
       <c r="AU37" s="2"/>
     </row>
-    <row r="38" ht="37.5" customHeight="1" spans="1:47">
+    <row r="38" ht="27.75" customHeight="1" spans="1:47">
       <c r="A38" s="20"/>
       <c r="B38" s="7"/>
       <c r="C38" s="20"/>
@@ -3740,7 +3671,7 @@
       <c r="AT40" s="7"/>
       <c r="AU40" s="2"/>
     </row>
-    <row r="41" ht="27.75" customHeight="1" spans="1:47">
+    <row r="41" ht="46.5" customHeight="1" spans="1:47">
       <c r="A41" s="20"/>
       <c r="B41" s="7"/>
       <c r="C41" s="20"/>
@@ -3789,7 +3720,7 @@
       <c r="AT41" s="7"/>
       <c r="AU41" s="2"/>
     </row>
-    <row r="42" ht="46.5" customHeight="1" spans="1:47">
+    <row r="42" ht="27.75" customHeight="1" spans="1:47">
       <c r="A42" s="20"/>
       <c r="B42" s="7"/>
       <c r="C42" s="20"/>
@@ -3838,7 +3769,7 @@
       <c r="AT42" s="7"/>
       <c r="AU42" s="2"/>
     </row>
-    <row r="43" ht="27.75" customHeight="1" spans="1:47">
+    <row r="43" ht="37.5" customHeight="1" spans="1:47">
       <c r="A43" s="20"/>
       <c r="B43" s="7"/>
       <c r="C43" s="20"/>
@@ -3887,7 +3818,7 @@
       <c r="AT43" s="7"/>
       <c r="AU43" s="2"/>
     </row>
-    <row r="44" ht="37.5" customHeight="1" spans="1:47">
+    <row r="44" ht="27.75" customHeight="1" spans="1:47">
       <c r="A44" s="20"/>
       <c r="B44" s="7"/>
       <c r="C44" s="20"/>
@@ -3936,7 +3867,7 @@
       <c r="AT44" s="7"/>
       <c r="AU44" s="2"/>
     </row>
-    <row r="45" ht="27.75" customHeight="1" spans="1:47">
+    <row r="45" ht="46.5" customHeight="1" spans="1:47">
       <c r="A45" s="20"/>
       <c r="B45" s="7"/>
       <c r="C45" s="20"/>
@@ -3985,7 +3916,7 @@
       <c r="AT45" s="7"/>
       <c r="AU45" s="2"/>
     </row>
-    <row r="46" ht="46.5" customHeight="1" spans="1:47">
+    <row r="46" ht="27.75" customHeight="1" spans="1:47">
       <c r="A46" s="20"/>
       <c r="B46" s="7"/>
       <c r="C46" s="20"/>
@@ -4034,7 +3965,7 @@
       <c r="AT46" s="7"/>
       <c r="AU46" s="2"/>
     </row>
-    <row r="47" ht="27.75" customHeight="1" spans="1:47">
+    <row r="47" ht="37.5" customHeight="1" spans="1:47">
       <c r="A47" s="20"/>
       <c r="B47" s="7"/>
       <c r="C47" s="20"/>
@@ -4181,7 +4112,7 @@
       <c r="AT49" s="7"/>
       <c r="AU49" s="2"/>
     </row>
-    <row r="50" ht="37.5" customHeight="1" spans="1:47">
+    <row r="50" ht="27.75" customHeight="1" spans="1:47">
       <c r="A50" s="20"/>
       <c r="B50" s="7"/>
       <c r="C50" s="20"/>
@@ -4230,7 +4161,7 @@
       <c r="AT50" s="7"/>
       <c r="AU50" s="2"/>
     </row>
-    <row r="51" ht="27.75" customHeight="1" spans="1:47">
+    <row r="51" ht="37.5" customHeight="1" spans="1:47">
       <c r="A51" s="20"/>
       <c r="B51" s="7"/>
       <c r="C51" s="20"/>
@@ -4279,7 +4210,7 @@
       <c r="AT51" s="7"/>
       <c r="AU51" s="2"/>
     </row>
-    <row r="52" ht="37.5" customHeight="1" spans="1:47">
+    <row r="52" ht="27.75" customHeight="1" spans="1:47">
       <c r="A52" s="20"/>
       <c r="B52" s="7"/>
       <c r="C52" s="20"/>
@@ -4426,7 +4357,7 @@
       <c r="AT54" s="7"/>
       <c r="AU54" s="2"/>
     </row>
-    <row r="55" ht="27.75" customHeight="1" spans="1:47">
+    <row r="55" ht="37.5" customHeight="1" spans="1:47">
       <c r="A55" s="20"/>
       <c r="B55" s="7"/>
       <c r="C55" s="20"/>
@@ -4475,7 +4406,7 @@
       <c r="AT55" s="7"/>
       <c r="AU55" s="2"/>
     </row>
-    <row r="56" ht="37.5" customHeight="1" spans="1:47">
+    <row r="56" ht="27.75" customHeight="1" spans="1:47">
       <c r="A56" s="20"/>
       <c r="B56" s="7"/>
       <c r="C56" s="20"/>
@@ -4524,336 +4455,207 @@
       <c r="AT56" s="7"/>
       <c r="AU56" s="2"/>
     </row>
-    <row r="57" ht="27.75" customHeight="1" spans="1:47">
-      <c r="A57" s="20"/>
-      <c r="B57" s="7"/>
-      <c r="C57" s="20"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="6"/>
-      <c r="F57" s="7"/>
-      <c r="G57" s="21"/>
-      <c r="H57" s="22"/>
-      <c r="I57" s="7"/>
-      <c r="J57" s="23"/>
-      <c r="K57" s="7"/>
-      <c r="L57" s="20"/>
-      <c r="M57" s="7"/>
-      <c r="N57" s="24"/>
-      <c r="O57" s="24"/>
-      <c r="P57" s="20"/>
-      <c r="Q57" s="7"/>
-      <c r="R57" s="20"/>
-      <c r="S57" s="6"/>
-      <c r="T57" s="7"/>
-      <c r="U57" s="20"/>
-      <c r="V57" s="7"/>
-      <c r="W57" s="20"/>
-      <c r="X57" s="6"/>
-      <c r="Y57" s="6"/>
-      <c r="Z57" s="6"/>
-      <c r="AA57" s="7"/>
-      <c r="AB57" s="20"/>
-      <c r="AC57" s="6"/>
-      <c r="AD57" s="6"/>
-      <c r="AE57" s="7"/>
-      <c r="AF57" s="20"/>
-      <c r="AG57" s="6"/>
-      <c r="AH57" s="6"/>
-      <c r="AI57" s="6"/>
-      <c r="AJ57" s="7"/>
-      <c r="AK57" s="20"/>
-      <c r="AL57" s="6"/>
-      <c r="AM57" s="6"/>
-      <c r="AN57" s="7"/>
-      <c r="AO57" s="24"/>
-      <c r="AP57" s="25"/>
-      <c r="AQ57" s="7"/>
-      <c r="AR57" s="21"/>
-      <c r="AS57" s="23"/>
-      <c r="AT57" s="7"/>
+    <row r="57" customHeight="1" spans="1:47">
+      <c r="A57" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="T57" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="V57" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="AT57" s="2"/>
       <c r="AU57" s="2"/>
     </row>
-    <row r="58" ht="19.5" customHeight="1" spans="1:47">
-      <c r="A58" s="26"/>
-      <c r="B58" s="7"/>
-      <c r="C58" s="20" t="s">
+    <row r="58" customHeight="1" spans="1:47">
+      <c r="A58" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="D58" s="6"/>
+      <c r="B58" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C58" s="7"/>
+      <c r="D58" s="30" t="s">
+        <v>38</v>
+      </c>
       <c r="E58" s="6"/>
-      <c r="F58" s="7"/>
-      <c r="G58" s="27" t="s">
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="J58" s="6"/>
+      <c r="K58" s="6"/>
+      <c r="L58" s="7"/>
+      <c r="M58" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="N58" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="O58" s="6"/>
+      <c r="P58" s="6"/>
+      <c r="Q58" s="6"/>
+      <c r="R58" s="6"/>
+      <c r="S58" s="7"/>
+      <c r="V58" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="W58" s="7"/>
+      <c r="X58" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y58" s="6"/>
+      <c r="Z58" s="7"/>
+      <c r="AA58" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB58" s="7"/>
+      <c r="AC58" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="H58" s="28" t="s">
+      <c r="AE58" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="AL58" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="I58" s="7"/>
-      <c r="J58" s="29" t="s">
+      <c r="AN58" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="AT58" s="2"/>
+      <c r="AU58" s="2"/>
+    </row>
+    <row r="59" ht="13.5" customHeight="1" spans="1:47">
+      <c r="A59" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="B59" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="C59" s="9"/>
+      <c r="D59" s="34" t="s">
+        <v>46</v>
+      </c>
+      <c r="E59" s="10"/>
+      <c r="F59" s="10"/>
+      <c r="G59" s="10"/>
+      <c r="H59" s="9"/>
+      <c r="I59" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="J59" s="10"/>
+      <c r="K59" s="10"/>
+      <c r="L59" s="9"/>
+      <c r="M59" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="N59" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="O59" s="10"/>
+      <c r="P59" s="10"/>
+      <c r="Q59" s="10"/>
+      <c r="R59" s="10"/>
+      <c r="S59" s="9"/>
+      <c r="V59" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="W59" s="9"/>
+      <c r="X59" s="8">
+        <v>25</v>
+      </c>
+      <c r="Y59" s="10"/>
+      <c r="Z59" s="9"/>
+      <c r="AA59" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="K58" s="7"/>
-      <c r="L58" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="M58" s="7"/>
-      <c r="N58" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="O58" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="P58" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q58" s="7"/>
-      <c r="R58" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="S58" s="6"/>
-      <c r="T58" s="7"/>
-      <c r="U58" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="V58" s="7"/>
-      <c r="W58" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="X58" s="6"/>
-      <c r="Y58" s="6"/>
-      <c r="Z58" s="6"/>
-      <c r="AA58" s="7"/>
-      <c r="AB58" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC58" s="6"/>
-      <c r="AD58" s="6"/>
-      <c r="AE58" s="7"/>
-      <c r="AF58" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG58" s="6"/>
-      <c r="AH58" s="6"/>
-      <c r="AI58" s="6"/>
-      <c r="AJ58" s="7"/>
-      <c r="AK58" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL58" s="6"/>
-      <c r="AM58" s="6"/>
-      <c r="AN58" s="7"/>
-      <c r="AO58" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AP58" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AQ58" s="7"/>
-      <c r="AR58" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AS58" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AT58" s="7"/>
-      <c r="AU58" s="2"/>
-    </row>
-    <row r="59" ht="19.5" customHeight="1" spans="1:47">
-      <c r="A59" s="26"/>
-      <c r="B59" s="7"/>
-      <c r="C59" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6"/>
-      <c r="F59" s="7"/>
-      <c r="G59" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="H59" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="I59" s="7"/>
-      <c r="J59" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="K59" s="7"/>
-      <c r="L59" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="M59" s="7"/>
-      <c r="N59" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="O59" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="P59" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q59" s="7"/>
-      <c r="R59" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="S59" s="6"/>
-      <c r="T59" s="7"/>
-      <c r="U59" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="V59" s="7"/>
-      <c r="W59" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="X59" s="6"/>
-      <c r="Y59" s="6"/>
-      <c r="Z59" s="6"/>
-      <c r="AA59" s="7"/>
-      <c r="AB59" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="AC59" s="6"/>
-      <c r="AD59" s="6"/>
-      <c r="AE59" s="7"/>
-      <c r="AF59" s="29" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG59" s="6"/>
-      <c r="AH59" s="6"/>
-      <c r="AI59" s="6"/>
-      <c r="AJ59" s="7"/>
-      <c r="AK59" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL59" s="6"/>
-      <c r="AM59" s="6"/>
-      <c r="AN59" s="7"/>
-      <c r="AO59" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AP59" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AQ59" s="7"/>
-      <c r="AR59" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="AS59" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="AT59" s="7"/>
+      <c r="AB59" s="9"/>
+      <c r="AE59" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="AN59" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="AT59" s="2"/>
       <c r="AU59" s="2"/>
     </row>
-    <row r="60" customHeight="1" spans="1:47">
-      <c r="A60" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="T60" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="V60" s="34" t="s">
-        <v>35</v>
-      </c>
+    <row r="60" ht="0.75" customHeight="1" spans="1:47">
+      <c r="A60" s="38"/>
+      <c r="B60" s="39"/>
+      <c r="C60" s="40"/>
+      <c r="D60" s="39"/>
+      <c r="H60" s="40"/>
+      <c r="I60" s="39"/>
+      <c r="L60" s="40"/>
+      <c r="M60" s="38"/>
+      <c r="N60" s="39"/>
+      <c r="S60" s="40"/>
+      <c r="V60" s="39"/>
+      <c r="W60" s="40"/>
+      <c r="X60" s="39"/>
+      <c r="Z60" s="40"/>
+      <c r="AA60" s="39"/>
+      <c r="AB60" s="40"/>
+      <c r="AN60" s="2"/>
+      <c r="AO60" s="2"/>
+      <c r="AP60" s="2"/>
+      <c r="AQ60" s="2"/>
+      <c r="AR60" s="2"/>
+      <c r="AS60" s="2"/>
       <c r="AT60" s="2"/>
       <c r="AU60" s="2"/>
     </row>
-    <row r="61" customHeight="1" spans="1:47">
-      <c r="A61" s="35" t="s">
-        <v>39</v>
-      </c>
-      <c r="B61" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C61" s="7"/>
-      <c r="D61" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="E61" s="6"/>
-      <c r="F61" s="6"/>
-      <c r="G61" s="6"/>
-      <c r="H61" s="7"/>
-      <c r="I61" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="J61" s="6"/>
-      <c r="K61" s="6"/>
-      <c r="L61" s="7"/>
-      <c r="M61" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="N61" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="O61" s="6"/>
-      <c r="P61" s="6"/>
-      <c r="Q61" s="6"/>
-      <c r="R61" s="6"/>
-      <c r="S61" s="7"/>
-      <c r="V61" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="W61" s="7"/>
-      <c r="X61" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="Y61" s="6"/>
-      <c r="Z61" s="7"/>
-      <c r="AA61" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="AB61" s="7"/>
-      <c r="AC61" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="AE61" s="37" t="s">
-        <v>45</v>
-      </c>
-      <c r="AL61" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="AN61" s="37" t="s">
-        <v>46</v>
+    <row r="61" ht="9.75" customHeight="1" spans="1:47">
+      <c r="A61" s="38"/>
+      <c r="B61" s="39"/>
+      <c r="C61" s="40"/>
+      <c r="D61" s="39"/>
+      <c r="H61" s="40"/>
+      <c r="I61" s="39"/>
+      <c r="L61" s="40"/>
+      <c r="M61" s="38"/>
+      <c r="N61" s="39"/>
+      <c r="S61" s="40"/>
+      <c r="V61" s="15"/>
+      <c r="W61" s="16"/>
+      <c r="X61" s="15"/>
+      <c r="Y61" s="17"/>
+      <c r="Z61" s="16"/>
+      <c r="AA61" s="15"/>
+      <c r="AB61" s="16"/>
+      <c r="AE61" s="41"/>
+      <c r="AF61" s="41"/>
+      <c r="AG61" s="41"/>
+      <c r="AH61" s="41"/>
+      <c r="AI61" s="41"/>
+      <c r="AJ61" s="41"/>
+      <c r="AK61" s="41"/>
+      <c r="AN61" s="42" t="s">
+        <v>53</v>
       </c>
       <c r="AT61" s="2"/>
       <c r="AU61" s="2"/>
     </row>
-    <row r="62" ht="13.5" customHeight="1" spans="1:47">
-      <c r="A62" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="B62" s="39" t="s">
-        <v>48</v>
-      </c>
-      <c r="C62" s="9"/>
-      <c r="D62" s="40" t="s">
-        <v>49</v>
-      </c>
-      <c r="E62" s="10"/>
-      <c r="F62" s="10"/>
-      <c r="G62" s="10"/>
-      <c r="H62" s="9"/>
-      <c r="I62" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="J62" s="10"/>
-      <c r="K62" s="10"/>
-      <c r="L62" s="9"/>
-      <c r="M62" s="41" t="s">
-        <v>51</v>
-      </c>
-      <c r="N62" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="O62" s="10"/>
-      <c r="P62" s="10"/>
-      <c r="Q62" s="10"/>
-      <c r="R62" s="10"/>
-      <c r="S62" s="9"/>
+    <row r="62" ht="9.75" customHeight="1" spans="1:47">
+      <c r="A62" s="38"/>
+      <c r="B62" s="39"/>
+      <c r="C62" s="40"/>
+      <c r="D62" s="39"/>
+      <c r="H62" s="40"/>
+      <c r="I62" s="39"/>
+      <c r="L62" s="40"/>
+      <c r="M62" s="38"/>
+      <c r="N62" s="39"/>
+      <c r="S62" s="40"/>
       <c r="V62" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="W62" s="9"/>
       <c r="X62" s="8">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Y62" s="10"/>
       <c r="Z62" s="9"/>
@@ -4862,201 +4664,222 @@
       </c>
       <c r="AB62" s="9"/>
       <c r="AE62" s="42" t="s">
-        <v>54</v>
-      </c>
-      <c r="AN62" s="43" t="s">
         <v>55</v>
       </c>
       <c r="AT62" s="2"/>
       <c r="AU62" s="2"/>
     </row>
-    <row r="63" ht="0.75" customHeight="1" spans="1:47">
-      <c r="A63" s="44"/>
-      <c r="B63" s="45"/>
-      <c r="C63" s="46"/>
-      <c r="D63" s="45"/>
-      <c r="H63" s="46"/>
-      <c r="I63" s="45"/>
-      <c r="L63" s="46"/>
-      <c r="M63" s="44"/>
-      <c r="N63" s="45"/>
-      <c r="S63" s="46"/>
-      <c r="V63" s="45"/>
-      <c r="W63" s="46"/>
-      <c r="X63" s="45"/>
-      <c r="Z63" s="46"/>
-      <c r="AA63" s="45"/>
-      <c r="AB63" s="46"/>
-      <c r="AN63" s="2"/>
-      <c r="AO63" s="2"/>
-      <c r="AP63" s="2"/>
-      <c r="AQ63" s="2"/>
-      <c r="AR63" s="2"/>
-      <c r="AS63" s="2"/>
+    <row r="63" ht="9.75" customHeight="1" spans="1:47">
+      <c r="A63" s="38"/>
+      <c r="B63" s="39"/>
+      <c r="C63" s="40"/>
+      <c r="D63" s="39"/>
+      <c r="H63" s="40"/>
+      <c r="I63" s="39"/>
+      <c r="L63" s="40"/>
+      <c r="M63" s="38"/>
+      <c r="N63" s="39"/>
+      <c r="S63" s="40"/>
+      <c r="V63" s="15"/>
+      <c r="W63" s="16"/>
+      <c r="X63" s="15"/>
+      <c r="Y63" s="17"/>
+      <c r="Z63" s="16"/>
+      <c r="AA63" s="15"/>
+      <c r="AB63" s="16"/>
+      <c r="AN63" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="AQ63" s="43" t="s">
+        <v>57</v>
+      </c>
       <c r="AT63" s="2"/>
       <c r="AU63" s="2"/>
     </row>
     <row r="64" ht="9.75" customHeight="1" spans="1:47">
-      <c r="A64" s="44"/>
-      <c r="B64" s="45"/>
-      <c r="C64" s="46"/>
-      <c r="D64" s="45"/>
-      <c r="H64" s="46"/>
-      <c r="I64" s="45"/>
-      <c r="L64" s="46"/>
-      <c r="M64" s="44"/>
-      <c r="N64" s="45"/>
-      <c r="S64" s="46"/>
-      <c r="V64" s="15"/>
-      <c r="W64" s="16"/>
-      <c r="X64" s="15"/>
-      <c r="Y64" s="17"/>
-      <c r="Z64" s="16"/>
-      <c r="AA64" s="15"/>
-      <c r="AB64" s="16"/>
-      <c r="AE64" s="47"/>
-      <c r="AF64" s="47"/>
-      <c r="AG64" s="47"/>
-      <c r="AH64" s="47"/>
-      <c r="AI64" s="47"/>
-      <c r="AJ64" s="47"/>
-      <c r="AK64" s="47"/>
-      <c r="AN64" s="48" t="s">
+      <c r="A64" s="38"/>
+      <c r="B64" s="39"/>
+      <c r="C64" s="40"/>
+      <c r="D64" s="39"/>
+      <c r="H64" s="40"/>
+      <c r="I64" s="39"/>
+      <c r="L64" s="40"/>
+      <c r="M64" s="38"/>
+      <c r="N64" s="39"/>
+      <c r="S64" s="40"/>
+      <c r="V64" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="W64" s="9"/>
+      <c r="X64" s="8">
+        <v>51</v>
+      </c>
+      <c r="Y64" s="10"/>
+      <c r="Z64" s="9"/>
+      <c r="AA64" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB64" s="9"/>
+      <c r="AE64" s="43" t="s">
         <v>56</v>
       </c>
+      <c r="AI64" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="AN64" s="41"/>
+      <c r="AO64" s="41"/>
+      <c r="AP64" s="41"/>
+      <c r="AQ64" s="41"/>
+      <c r="AR64" s="41"/>
+      <c r="AS64" s="41"/>
       <c r="AT64" s="2"/>
       <c r="AU64" s="2"/>
     </row>
-    <row r="65" ht="9.75" customHeight="1" spans="1:47">
-      <c r="A65" s="44"/>
-      <c r="B65" s="45"/>
-      <c r="C65" s="46"/>
-      <c r="D65" s="45"/>
-      <c r="H65" s="46"/>
-      <c r="I65" s="45"/>
-      <c r="L65" s="46"/>
-      <c r="M65" s="44"/>
-      <c r="N65" s="45"/>
-      <c r="S65" s="46"/>
-      <c r="V65" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="W65" s="9"/>
-      <c r="X65" s="8">
-        <v>26</v>
-      </c>
-      <c r="Y65" s="10"/>
-      <c r="Z65" s="9"/>
-      <c r="AA65" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB65" s="9"/>
-      <c r="AE65" s="48" t="s">
-        <v>58</v>
-      </c>
+    <row r="65" customHeight="1" spans="1:47">
+      <c r="A65" s="18"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="16"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="17"/>
+      <c r="F65" s="17"/>
+      <c r="G65" s="17"/>
+      <c r="H65" s="16"/>
+      <c r="I65" s="15"/>
+      <c r="J65" s="17"/>
+      <c r="K65" s="17"/>
+      <c r="L65" s="16"/>
+      <c r="M65" s="18"/>
+      <c r="N65" s="15"/>
+      <c r="O65" s="17"/>
+      <c r="P65" s="17"/>
+      <c r="Q65" s="17"/>
+      <c r="R65" s="17"/>
+      <c r="S65" s="16"/>
+      <c r="V65" s="15"/>
+      <c r="W65" s="16"/>
+      <c r="X65" s="15"/>
+      <c r="Y65" s="17"/>
+      <c r="Z65" s="16"/>
+      <c r="AA65" s="15"/>
+      <c r="AB65" s="16"/>
+      <c r="AE65" s="41"/>
+      <c r="AF65" s="41"/>
+      <c r="AG65" s="41"/>
+      <c r="AH65" s="41"/>
+      <c r="AI65" s="41"/>
+      <c r="AJ65" s="41"/>
+      <c r="AK65" s="41"/>
+      <c r="AN65" s="2"/>
+      <c r="AO65" s="2"/>
+      <c r="AP65" s="2"/>
+      <c r="AQ65" s="2"/>
+      <c r="AR65" s="2"/>
+      <c r="AS65" s="2"/>
       <c r="AT65" s="2"/>
       <c r="AU65" s="2"/>
     </row>
     <row r="66" ht="9.75" customHeight="1" spans="1:47">
-      <c r="A66" s="44"/>
-      <c r="B66" s="45"/>
-      <c r="C66" s="46"/>
-      <c r="D66" s="45"/>
-      <c r="H66" s="46"/>
-      <c r="I66" s="45"/>
-      <c r="L66" s="46"/>
-      <c r="M66" s="44"/>
-      <c r="N66" s="45"/>
-      <c r="S66" s="46"/>
-      <c r="V66" s="15"/>
-      <c r="W66" s="16"/>
-      <c r="X66" s="15"/>
-      <c r="Y66" s="17"/>
-      <c r="Z66" s="16"/>
-      <c r="AA66" s="15"/>
-      <c r="AB66" s="16"/>
-      <c r="AN66" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="AQ66" s="49" t="s">
-        <v>60</v>
-      </c>
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
+      <c r="G66" s="2"/>
+      <c r="H66" s="2"/>
+      <c r="I66" s="2"/>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
+      <c r="L66" s="2"/>
+      <c r="M66" s="2"/>
+      <c r="N66" s="2"/>
+      <c r="O66" s="2"/>
+      <c r="P66" s="2"/>
+      <c r="Q66" s="2"/>
+      <c r="R66" s="2"/>
+      <c r="S66" s="2"/>
+      <c r="T66" s="2"/>
+      <c r="U66" s="2"/>
+      <c r="V66" s="2"/>
+      <c r="W66" s="2"/>
+      <c r="X66" s="2"/>
+      <c r="Y66" s="2"/>
+      <c r="Z66" s="2"/>
+      <c r="AA66" s="2"/>
+      <c r="AB66" s="2"/>
+      <c r="AC66" s="2"/>
+      <c r="AD66" s="2"/>
+      <c r="AE66" s="2"/>
+      <c r="AF66" s="2"/>
+      <c r="AG66" s="2"/>
+      <c r="AH66" s="2"/>
+      <c r="AI66" s="2"/>
+      <c r="AJ66" s="2"/>
+      <c r="AK66" s="2"/>
+      <c r="AN66" s="2"/>
+      <c r="AO66" s="2"/>
+      <c r="AP66" s="2"/>
+      <c r="AQ66" s="2"/>
+      <c r="AR66" s="2"/>
+      <c r="AS66" s="2"/>
       <c r="AT66" s="2"/>
       <c r="AU66" s="2"/>
     </row>
     <row r="67" ht="9.75" customHeight="1" spans="1:47">
-      <c r="A67" s="44"/>
-      <c r="B67" s="45"/>
-      <c r="C67" s="46"/>
-      <c r="D67" s="45"/>
-      <c r="H67" s="46"/>
-      <c r="I67" s="45"/>
-      <c r="L67" s="46"/>
-      <c r="M67" s="44"/>
-      <c r="N67" s="45"/>
-      <c r="S67" s="46"/>
-      <c r="V67" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="W67" s="9"/>
-      <c r="X67" s="8">
-        <v>51</v>
-      </c>
-      <c r="Y67" s="10"/>
-      <c r="Z67" s="9"/>
-      <c r="AA67" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="AB67" s="9"/>
-      <c r="AE67" s="49" t="s">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
+      <c r="F67" s="2"/>
+      <c r="G67" s="2"/>
+      <c r="H67" s="2"/>
+      <c r="I67" s="2"/>
+      <c r="J67" s="2"/>
+      <c r="K67" s="2"/>
+      <c r="L67" s="2"/>
+      <c r="M67" s="2"/>
+      <c r="N67" s="2"/>
+      <c r="O67" s="2"/>
+      <c r="P67" s="2"/>
+      <c r="Q67" s="2"/>
+      <c r="R67" s="2"/>
+      <c r="S67" s="2"/>
+      <c r="T67" s="2"/>
+      <c r="U67" s="2"/>
+      <c r="V67" s="2"/>
+      <c r="W67" s="2"/>
+      <c r="X67" s="2"/>
+      <c r="Y67" s="2"/>
+      <c r="Z67" s="2"/>
+      <c r="AA67" s="2"/>
+      <c r="AB67" s="2"/>
+      <c r="AC67" s="2"/>
+      <c r="AD67" s="2"/>
+      <c r="AE67" s="2"/>
+      <c r="AF67" s="2"/>
+      <c r="AG67" s="2"/>
+      <c r="AH67" s="2"/>
+      <c r="AI67" s="2"/>
+      <c r="AJ67" s="2"/>
+      <c r="AK67" s="2"/>
+      <c r="AN67" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="AI67" s="49" t="s">
-        <v>60</v>
-      </c>
-      <c r="AN67" s="47"/>
-      <c r="AO67" s="47"/>
-      <c r="AP67" s="47"/>
-      <c r="AQ67" s="47"/>
-      <c r="AR67" s="47"/>
-      <c r="AS67" s="47"/>
+      <c r="AO67" s="45"/>
+      <c r="AP67" s="45"/>
+      <c r="AQ67" s="45"/>
+      <c r="AR67" s="45"/>
+      <c r="AS67" s="45"/>
       <c r="AT67" s="2"/>
       <c r="AU67" s="2"/>
     </row>
-    <row r="68" customHeight="1" spans="1:47">
-      <c r="A68" s="18"/>
-      <c r="B68" s="15"/>
-      <c r="C68" s="16"/>
-      <c r="D68" s="15"/>
-      <c r="E68" s="17"/>
-      <c r="F68" s="17"/>
-      <c r="G68" s="17"/>
-      <c r="H68" s="16"/>
-      <c r="I68" s="15"/>
-      <c r="J68" s="17"/>
-      <c r="K68" s="17"/>
-      <c r="L68" s="16"/>
-      <c r="M68" s="18"/>
-      <c r="N68" s="15"/>
-      <c r="O68" s="17"/>
-      <c r="P68" s="17"/>
-      <c r="Q68" s="17"/>
-      <c r="R68" s="17"/>
-      <c r="S68" s="16"/>
-      <c r="V68" s="15"/>
-      <c r="W68" s="16"/>
-      <c r="X68" s="15"/>
-      <c r="Y68" s="17"/>
-      <c r="Z68" s="16"/>
-      <c r="AA68" s="15"/>
-      <c r="AB68" s="16"/>
-      <c r="AE68" s="47"/>
-      <c r="AF68" s="47"/>
-      <c r="AG68" s="47"/>
-      <c r="AH68" s="47"/>
-      <c r="AI68" s="47"/>
-      <c r="AJ68" s="47"/>
-      <c r="AK68" s="47"/>
+    <row r="68" ht="19.5" customHeight="1" spans="1:47">
+      <c r="A68" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL68" s="2"/>
+      <c r="AM68" s="2"/>
       <c r="AN68" s="2"/>
       <c r="AO68" s="2"/>
       <c r="AP68" s="2"/>
@@ -5066,117 +4889,9 @@
       <c r="AT68" s="2"/>
       <c r="AU68" s="2"/>
     </row>
-    <row r="69" ht="9.75" customHeight="1" spans="1:47">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
-      <c r="G69" s="2"/>
-      <c r="H69" s="2"/>
-      <c r="I69" s="2"/>
-      <c r="J69" s="2"/>
-      <c r="K69" s="2"/>
-      <c r="L69" s="2"/>
-      <c r="M69" s="2"/>
-      <c r="N69" s="2"/>
-      <c r="O69" s="2"/>
-      <c r="P69" s="2"/>
-      <c r="Q69" s="2"/>
-      <c r="R69" s="2"/>
-      <c r="S69" s="2"/>
-      <c r="T69" s="2"/>
-      <c r="U69" s="2"/>
-      <c r="V69" s="2"/>
-      <c r="W69" s="2"/>
-      <c r="X69" s="2"/>
-      <c r="Y69" s="2"/>
-      <c r="Z69" s="2"/>
-      <c r="AA69" s="2"/>
-      <c r="AB69" s="2"/>
-      <c r="AC69" s="2"/>
-      <c r="AD69" s="2"/>
-      <c r="AE69" s="2"/>
-      <c r="AF69" s="2"/>
-      <c r="AG69" s="2"/>
-      <c r="AH69" s="2"/>
-      <c r="AI69" s="2"/>
-      <c r="AJ69" s="2"/>
-      <c r="AK69" s="2"/>
-      <c r="AN69" s="2"/>
-      <c r="AO69" s="2"/>
-      <c r="AP69" s="2"/>
-      <c r="AQ69" s="2"/>
-      <c r="AR69" s="2"/>
-      <c r="AS69" s="2"/>
-      <c r="AT69" s="2"/>
-      <c r="AU69" s="2"/>
-    </row>
-    <row r="70" ht="9.75" customHeight="1" spans="1:47">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
-      <c r="F70" s="2"/>
-      <c r="G70" s="2"/>
-      <c r="H70" s="2"/>
-      <c r="I70" s="2"/>
-      <c r="J70" s="2"/>
-      <c r="K70" s="2"/>
-      <c r="L70" s="2"/>
-      <c r="M70" s="2"/>
-      <c r="N70" s="2"/>
-      <c r="O70" s="2"/>
-      <c r="P70" s="2"/>
-      <c r="Q70" s="2"/>
-      <c r="R70" s="2"/>
-      <c r="S70" s="2"/>
-      <c r="T70" s="2"/>
-      <c r="U70" s="2"/>
-      <c r="V70" s="2"/>
-      <c r="W70" s="2"/>
-      <c r="X70" s="2"/>
-      <c r="Y70" s="2"/>
-      <c r="Z70" s="2"/>
-      <c r="AA70" s="2"/>
-      <c r="AB70" s="2"/>
-      <c r="AC70" s="2"/>
-      <c r="AD70" s="2"/>
-      <c r="AE70" s="2"/>
-      <c r="AF70" s="2"/>
-      <c r="AG70" s="2"/>
-      <c r="AH70" s="2"/>
-      <c r="AI70" s="2"/>
-      <c r="AJ70" s="2"/>
-      <c r="AK70" s="2"/>
-      <c r="AN70" s="50" t="s">
-        <v>62</v>
-      </c>
-      <c r="AO70" s="51"/>
-      <c r="AP70" s="51"/>
-      <c r="AQ70" s="51"/>
-      <c r="AR70" s="51"/>
-      <c r="AS70" s="51"/>
-      <c r="AT70" s="2"/>
-      <c r="AU70" s="2"/>
-    </row>
-    <row r="71" ht="19.5" customHeight="1" spans="1:47">
-      <c r="A71" s="52" t="s">
-        <v>63</v>
-      </c>
-      <c r="AL71" s="2"/>
-      <c r="AM71" s="2"/>
-      <c r="AN71" s="2"/>
-      <c r="AO71" s="2"/>
-      <c r="AP71" s="2"/>
-      <c r="AQ71" s="2"/>
-      <c r="AR71" s="2"/>
-      <c r="AS71" s="2"/>
-      <c r="AT71" s="2"/>
-      <c r="AU71" s="2"/>
-    </row>
+    <row r="69" ht="12.75" customHeight="1"/>
+    <row r="70" ht="12.75" customHeight="1"/>
+    <row r="71" ht="12.75" customHeight="1"/>
     <row r="72" ht="12.75" customHeight="1"/>
     <row r="73" ht="12.75" customHeight="1"/>
     <row r="74" ht="12.75" customHeight="1"/>
@@ -6102,11 +5817,8 @@
     <row r="994" ht="12.75" customHeight="1"/>
     <row r="995" ht="12.75" customHeight="1"/>
     <row r="996" ht="12.75" customHeight="1"/>
-    <row r="997" ht="12.75" customHeight="1"/>
-    <row r="998" ht="12.75" customHeight="1"/>
-    <row r="999" ht="12.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="818">
+  <mergeCells count="776">
     <mergeCell ref="A1:AT1"/>
     <mergeCell ref="A2:AT2"/>
     <mergeCell ref="A3:E3"/>
@@ -6834,65 +6546,23 @@
     <mergeCell ref="AK56:AN56"/>
     <mergeCell ref="AP56:AQ56"/>
     <mergeCell ref="AS56:AT56"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="C57:F57"/>
-    <mergeCell ref="H57:I57"/>
-    <mergeCell ref="J57:K57"/>
-    <mergeCell ref="L57:M57"/>
-    <mergeCell ref="P57:Q57"/>
-    <mergeCell ref="R57:T57"/>
-    <mergeCell ref="U57:V57"/>
-    <mergeCell ref="W57:AA57"/>
-    <mergeCell ref="AB57:AE57"/>
-    <mergeCell ref="AF57:AJ57"/>
-    <mergeCell ref="AK57:AN57"/>
-    <mergeCell ref="AP57:AQ57"/>
-    <mergeCell ref="AS57:AT57"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="C58:F58"/>
-    <mergeCell ref="H58:I58"/>
-    <mergeCell ref="J58:K58"/>
-    <mergeCell ref="L58:M58"/>
-    <mergeCell ref="P58:Q58"/>
-    <mergeCell ref="R58:T58"/>
-    <mergeCell ref="U58:V58"/>
-    <mergeCell ref="W58:AA58"/>
-    <mergeCell ref="AB58:AE58"/>
-    <mergeCell ref="AF58:AJ58"/>
-    <mergeCell ref="AK58:AN58"/>
-    <mergeCell ref="AP58:AQ58"/>
-    <mergeCell ref="AS58:AT58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="C59:F59"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="J59:K59"/>
-    <mergeCell ref="L59:M59"/>
-    <mergeCell ref="P59:Q59"/>
-    <mergeCell ref="R59:T59"/>
-    <mergeCell ref="U59:V59"/>
-    <mergeCell ref="W59:AA59"/>
-    <mergeCell ref="AB59:AE59"/>
-    <mergeCell ref="AF59:AJ59"/>
-    <mergeCell ref="AK59:AN59"/>
-    <mergeCell ref="AP59:AQ59"/>
-    <mergeCell ref="AS59:AT59"/>
-    <mergeCell ref="A60:S60"/>
-    <mergeCell ref="V60:AS60"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="D61:H61"/>
-    <mergeCell ref="I61:L61"/>
-    <mergeCell ref="N61:S61"/>
-    <mergeCell ref="V61:W61"/>
-    <mergeCell ref="X61:Z61"/>
-    <mergeCell ref="AA61:AB61"/>
-    <mergeCell ref="AE61:AK61"/>
-    <mergeCell ref="AN61:AS61"/>
-    <mergeCell ref="AN62:AS62"/>
-    <mergeCell ref="AN70:AS70"/>
-    <mergeCell ref="A71:AK71"/>
-    <mergeCell ref="A62:A68"/>
+    <mergeCell ref="A57:S57"/>
+    <mergeCell ref="V57:AS57"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="D58:H58"/>
+    <mergeCell ref="I58:L58"/>
+    <mergeCell ref="N58:S58"/>
+    <mergeCell ref="V58:W58"/>
+    <mergeCell ref="X58:Z58"/>
+    <mergeCell ref="AA58:AB58"/>
+    <mergeCell ref="AE58:AK58"/>
+    <mergeCell ref="AN58:AS58"/>
+    <mergeCell ref="AN59:AS59"/>
+    <mergeCell ref="AN67:AS67"/>
+    <mergeCell ref="A68:AK68"/>
+    <mergeCell ref="A59:A65"/>
     <mergeCell ref="G5:G6"/>
-    <mergeCell ref="M62:M68"/>
+    <mergeCell ref="M59:M65"/>
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="O5:O6"/>
     <mergeCell ref="AR5:AR6"/>
@@ -6902,29 +6572,29 @@
     <mergeCell ref="AP5:AQ6"/>
     <mergeCell ref="A5:B6"/>
     <mergeCell ref="C5:F6"/>
-    <mergeCell ref="B62:C68"/>
-    <mergeCell ref="D62:H68"/>
-    <mergeCell ref="I62:L68"/>
-    <mergeCell ref="N62:S68"/>
-    <mergeCell ref="V62:W64"/>
-    <mergeCell ref="V65:W66"/>
-    <mergeCell ref="V67:W68"/>
-    <mergeCell ref="T60:U68"/>
-    <mergeCell ref="AE62:AK64"/>
-    <mergeCell ref="X65:Z66"/>
-    <mergeCell ref="AA65:AB66"/>
-    <mergeCell ref="AE65:AK66"/>
-    <mergeCell ref="AN66:AP67"/>
-    <mergeCell ref="AQ66:AS67"/>
-    <mergeCell ref="X62:Z64"/>
-    <mergeCell ref="X67:Z68"/>
-    <mergeCell ref="AA67:AB68"/>
-    <mergeCell ref="AE67:AH68"/>
-    <mergeCell ref="AC61:AD68"/>
-    <mergeCell ref="AL61:AM70"/>
-    <mergeCell ref="AA62:AB64"/>
-    <mergeCell ref="AI67:AK68"/>
-    <mergeCell ref="AN64:AS65"/>
+    <mergeCell ref="V64:W65"/>
+    <mergeCell ref="X64:Z65"/>
+    <mergeCell ref="AA64:AB65"/>
+    <mergeCell ref="B59:C65"/>
+    <mergeCell ref="D59:H65"/>
+    <mergeCell ref="I59:L65"/>
+    <mergeCell ref="N59:S65"/>
+    <mergeCell ref="V59:W61"/>
+    <mergeCell ref="V62:W63"/>
+    <mergeCell ref="T57:U65"/>
+    <mergeCell ref="AE59:AK61"/>
+    <mergeCell ref="X62:Z63"/>
+    <mergeCell ref="AA62:AB63"/>
+    <mergeCell ref="AE62:AK63"/>
+    <mergeCell ref="AN63:AP64"/>
+    <mergeCell ref="AQ63:AS64"/>
+    <mergeCell ref="X59:Z61"/>
+    <mergeCell ref="AE64:AH65"/>
+    <mergeCell ref="AC58:AD65"/>
+    <mergeCell ref="AL58:AM67"/>
+    <mergeCell ref="AA59:AB61"/>
+    <mergeCell ref="AI64:AK65"/>
+    <mergeCell ref="AN61:AS62"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="14" fitToHeight="0" orientation="landscape"/>

</xml_diff>

<commit_message>
feat(sf1): import and export school register
</commit_message>
<xml_diff>
--- a/backend/forms/SF1_template.xlsx
+++ b/backend/forms/SF1_template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
   <si>
     <t>School Form 1 (SF 1) School Register</t>
   </si>
@@ -202,12 +202,6 @@
   </si>
   <si>
     <t>MALE</t>
-  </si>
-  <si>
-    <t>CRIS IVY GUMBAN CAMPANAN</t>
-  </si>
-  <si>
-    <t>LOURDES ABELLA MONTEFRIO</t>
   </si>
   <si>
     <t>(Signature of School Head over Printed Name)</t>
@@ -4564,21 +4558,15 @@
         <v>50</v>
       </c>
       <c r="W59" s="9"/>
-      <c r="X59" s="8">
-        <v>25</v>
-      </c>
+      <c r="X59" s="8"/>
       <c r="Y59" s="10"/>
       <c r="Z59" s="9"/>
       <c r="AA59" s="8" t="s">
         <v>35</v>
       </c>
       <c r="AB59" s="9"/>
-      <c r="AE59" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="AN59" s="37" t="s">
-        <v>52</v>
-      </c>
+      <c r="AE59" s="36"/>
+      <c r="AN59" s="37"/>
       <c r="AT59" s="2"/>
       <c r="AU59" s="2"/>
     </row>
@@ -4634,7 +4622,7 @@
       <c r="AJ61" s="41"/>
       <c r="AK61" s="41"/>
       <c r="AN61" s="42" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="AT61" s="2"/>
       <c r="AU61" s="2"/>
@@ -4651,12 +4639,10 @@
       <c r="N62" s="39"/>
       <c r="S62" s="40"/>
       <c r="V62" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="W62" s="9"/>
-      <c r="X62" s="8">
-        <v>26</v>
-      </c>
+      <c r="X62" s="8"/>
       <c r="Y62" s="10"/>
       <c r="Z62" s="9"/>
       <c r="AA62" s="8" t="s">
@@ -4664,7 +4650,7 @@
       </c>
       <c r="AB62" s="9"/>
       <c r="AE62" s="42" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="AT62" s="2"/>
       <c r="AU62" s="2"/>
@@ -4688,10 +4674,10 @@
       <c r="AA63" s="15"/>
       <c r="AB63" s="16"/>
       <c r="AN63" s="43" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="AQ63" s="43" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="AT63" s="2"/>
       <c r="AU63" s="2"/>
@@ -4708,12 +4694,10 @@
       <c r="N64" s="39"/>
       <c r="S64" s="40"/>
       <c r="V64" s="8" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="W64" s="9"/>
-      <c r="X64" s="8">
-        <v>51</v>
-      </c>
+      <c r="X64" s="8"/>
       <c r="Y64" s="10"/>
       <c r="Z64" s="9"/>
       <c r="AA64" s="8" t="s">
@@ -4721,10 +4705,10 @@
       </c>
       <c r="AB64" s="9"/>
       <c r="AE64" s="43" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="AI64" s="43" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="AN64" s="41"/>
       <c r="AO64" s="41"/>
@@ -4864,7 +4848,7 @@
       <c r="AJ67" s="2"/>
       <c r="AK67" s="2"/>
       <c r="AN67" s="44" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="AO67" s="45"/>
       <c r="AP67" s="45"/>
@@ -4876,7 +4860,7 @@
     </row>
     <row r="68" ht="19.5" customHeight="1" spans="1:47">
       <c r="A68" s="46" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AL68" s="2"/>
       <c r="AM68" s="2"/>

</xml_diff>

<commit_message>
refactor(sf1-template): remove pre-filled school info
</commit_message>
<xml_diff>
--- a/backend/forms/SF1_template.xlsx
+++ b/backend/forms/SF1_template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
   <si>
     <t>School Form 1 (SF 1) School Register</t>
   </si>
@@ -38,19 +38,10 @@
     <t xml:space="preserve">School ID </t>
   </si>
   <si>
-    <t>Region VI</t>
-  </si>
-  <si>
     <t xml:space="preserve">Division </t>
   </si>
   <si>
-    <t>Iloilo</t>
-  </si>
-  <si>
     <t xml:space="preserve">School Name </t>
-  </si>
-  <si>
-    <t>Pavia National High School</t>
   </si>
   <si>
     <t xml:space="preserve">School Year </t>
@@ -1757,28 +1748,22 @@
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="5">
-        <v>302550</v>
-      </c>
+      <c r="F3" s="5"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
       <c r="I3" s="7"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="5" t="s">
-        <v>3</v>
-      </c>
+      <c r="K3" s="5"/>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
       <c r="O3" s="7"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S3" s="2"/>
-      <c r="T3" s="5" t="s">
-        <v>5</v>
-      </c>
+      <c r="T3" s="5"/>
       <c r="U3" s="6"/>
       <c r="V3" s="6"/>
       <c r="W3" s="6"/>
@@ -1809,11 +1794,9 @@
     </row>
     <row r="4" ht="19.5" customHeight="1" spans="1:47">
       <c r="A4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>7</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="F4" s="5"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
@@ -1825,7 +1808,7 @@
       <c r="O4" s="7"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="T4" s="5"/>
       <c r="U4" s="6"/>
@@ -1834,7 +1817,7 @@
       <c r="X4" s="7"/>
       <c r="Y4" s="2"/>
       <c r="Z4" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AD4" s="2"/>
       <c r="AE4" s="5"/>
@@ -1843,7 +1826,7 @@
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
       <c r="AJ4" s="4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="AM4" s="5"/>
       <c r="AN4" s="6"/>
@@ -1857,38 +1840,38 @@
     </row>
     <row r="5" ht="24.75" customHeight="1" spans="1:47">
       <c r="A5" s="8" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="8" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="9"/>
       <c r="G5" s="11" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I5" s="9"/>
       <c r="J5" s="12" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K5" s="9"/>
       <c r="L5" s="8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M5" s="9"/>
       <c r="N5" s="13" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="O5" s="13" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="P5" s="14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
@@ -1902,7 +1885,7 @@
       <c r="Z5" s="6"/>
       <c r="AA5" s="7"/>
       <c r="AB5" s="14" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AC5" s="6"/>
       <c r="AD5" s="6"/>
@@ -1913,21 +1896,21 @@
       <c r="AI5" s="6"/>
       <c r="AJ5" s="7"/>
       <c r="AK5" s="14" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="AL5" s="6"/>
       <c r="AM5" s="6"/>
       <c r="AN5" s="6"/>
       <c r="AO5" s="7"/>
       <c r="AP5" s="8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="AQ5" s="9"/>
       <c r="AR5" s="13" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AS5" s="14" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="AT5" s="7"/>
       <c r="AU5" s="2"/>
@@ -1949,52 +1932,52 @@
       <c r="N6" s="18"/>
       <c r="O6" s="18"/>
       <c r="P6" s="14" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="Q6" s="7"/>
       <c r="R6" s="14" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="S6" s="6"/>
       <c r="T6" s="7"/>
       <c r="U6" s="14" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="V6" s="7"/>
       <c r="W6" s="14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="X6" s="6"/>
       <c r="Y6" s="6"/>
       <c r="Z6" s="6"/>
       <c r="AA6" s="7"/>
       <c r="AB6" s="14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="AC6" s="6"/>
       <c r="AD6" s="6"/>
       <c r="AE6" s="7"/>
       <c r="AF6" s="14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="AG6" s="6"/>
       <c r="AH6" s="6"/>
       <c r="AI6" s="6"/>
       <c r="AJ6" s="7"/>
       <c r="AK6" s="14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="AL6" s="6"/>
       <c r="AM6" s="6"/>
       <c r="AN6" s="7"/>
       <c r="AO6" s="19" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="AP6" s="15"/>
       <c r="AQ6" s="16"/>
       <c r="AR6" s="18"/>
       <c r="AS6" s="14" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="AT6" s="7"/>
       <c r="AU6" s="2"/>
@@ -4451,43 +4434,43 @@
     </row>
     <row r="57" customHeight="1" spans="1:47">
       <c r="A57" s="26" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="T57" s="27" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="V57" s="28" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AT57" s="2"/>
       <c r="AU57" s="2"/>
     </row>
     <row r="58" customHeight="1" spans="1:47">
       <c r="A58" s="29" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C58" s="7"/>
       <c r="D58" s="30" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E58" s="6"/>
       <c r="F58" s="6"/>
       <c r="G58" s="6"/>
       <c r="H58" s="7"/>
       <c r="I58" s="30" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="J58" s="6"/>
       <c r="K58" s="6"/>
       <c r="L58" s="7"/>
       <c r="M58" s="19" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="N58" s="30" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="O58" s="6"/>
       <c r="P58" s="6"/>
@@ -4495,59 +4478,59 @@
       <c r="R58" s="6"/>
       <c r="S58" s="7"/>
       <c r="V58" s="14" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="W58" s="7"/>
       <c r="X58" s="14" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="Y58" s="6"/>
       <c r="Z58" s="7"/>
       <c r="AA58" s="14" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="AB58" s="7"/>
       <c r="AC58" s="27" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AE58" s="31" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="AL58" s="27" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AN58" s="31" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="AT58" s="2"/>
       <c r="AU58" s="2"/>
     </row>
     <row r="59" ht="13.5" customHeight="1" spans="1:47">
       <c r="A59" s="32" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B59" s="33" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="34" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E59" s="10"/>
       <c r="F59" s="10"/>
       <c r="G59" s="10"/>
       <c r="H59" s="9"/>
       <c r="I59" s="34" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J59" s="10"/>
       <c r="K59" s="10"/>
       <c r="L59" s="9"/>
       <c r="M59" s="35" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="N59" s="34" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="O59" s="10"/>
       <c r="P59" s="10"/>
@@ -4555,14 +4538,14 @@
       <c r="R59" s="10"/>
       <c r="S59" s="9"/>
       <c r="V59" s="8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="W59" s="9"/>
       <c r="X59" s="8"/>
       <c r="Y59" s="10"/>
       <c r="Z59" s="9"/>
       <c r="AA59" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AB59" s="9"/>
       <c r="AE59" s="36"/>
@@ -4622,7 +4605,7 @@
       <c r="AJ61" s="41"/>
       <c r="AK61" s="41"/>
       <c r="AN61" s="42" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="AT61" s="2"/>
       <c r="AU61" s="2"/>
@@ -4639,18 +4622,18 @@
       <c r="N62" s="39"/>
       <c r="S62" s="40"/>
       <c r="V62" s="8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="W62" s="9"/>
       <c r="X62" s="8"/>
       <c r="Y62" s="10"/>
       <c r="Z62" s="9"/>
       <c r="AA62" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AB62" s="9"/>
       <c r="AE62" s="42" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="AT62" s="2"/>
       <c r="AU62" s="2"/>
@@ -4674,10 +4657,10 @@
       <c r="AA63" s="15"/>
       <c r="AB63" s="16"/>
       <c r="AN63" s="43" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AQ63" s="43" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="AT63" s="2"/>
       <c r="AU63" s="2"/>
@@ -4694,21 +4677,21 @@
       <c r="N64" s="39"/>
       <c r="S64" s="40"/>
       <c r="V64" s="8" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="W64" s="9"/>
       <c r="X64" s="8"/>
       <c r="Y64" s="10"/>
       <c r="Z64" s="9"/>
       <c r="AA64" s="8" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="AB64" s="9"/>
       <c r="AE64" s="43" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AI64" s="43" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="AN64" s="41"/>
       <c r="AO64" s="41"/>
@@ -4848,7 +4831,7 @@
       <c r="AJ67" s="2"/>
       <c r="AK67" s="2"/>
       <c r="AN67" s="44" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="AO67" s="45"/>
       <c r="AP67" s="45"/>
@@ -4860,7 +4843,7 @@
     </row>
     <row r="68" ht="19.5" customHeight="1" spans="1:47">
       <c r="A68" s="46" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="AL68" s="2"/>
       <c r="AM68" s="2"/>

</xml_diff>